<commit_message>
MOTEUR_ELASTICITE : l'exposant redevient visible
Deux endroits ou la puissance ne se voyait plus :

- « La methode » affichait « ^ elasticite » depuis la passe precedente, un
  mot la ou on attend un nombre. La ligne est redevenue une formule vivante
  qui lit la pente du groupe : « ^ 0,46 ».

- Sur « Le moteur », POWER n'est present que sur les lignes CAMPUS — les
  lignes marque et groupe sont des sommes, par construction. La relation est
  maintenant ecrite en clair juste sous la cellule jaune, pour qu'on sache ou
  la chercher sans cliquer.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/MOTEUR_ELASTICITE.xlsx
+++ b/eduservices/MOTEUR_ELASTICITE.xlsx
@@ -1026,10 +1026,9 @@
           <t>inscrits 2027</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  =  inscrits 2026  ×  ( budget marketing 2027 ÷ budget marketing 2026 ) ^ élasticité</t>
-        </is>
+      <c r="D13" s="10">
+        <f>"  =  inscrits 2026  ×  ( budget marketing 2027 ÷ budget marketing 2026 ) ^ "&amp;TEXT(Historique!$M$25,"0.00")</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1190,6 +1189,13 @@
       <c r="E6" s="16" t="inlineStr">
         <is>
           <t>← le levier prix du cadrage V01</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Sur chaque ligne campus :  inscrits 2027  =  inscrits 2026  ×  ( 1 + Δ budget marketing ) ^ élasticité du campus.  Les lignes marque et la ligne groupe sont les sommes de leurs campus.</t>
         </is>
       </c>
     </row>

</xml_diff>